<commit_message>
Bulk-import remaining site pages; make block selectors resilient
Import the 10 non-representative pages across templates (2 landing, 2
listing, 6 blog articles) and switch landing-page + article-listing block
selectors from position-based (:nth-of-type) to class-based so all sections
are captured regardless of section order.

- landing-page + article-listing block instances now class-based; distinguishing
  classes preserved to avoid cross-block collisions
- article-listing gains cards-gallery/tabs-team/hero-overlay (some listing
  pages carry those sections)
- expanded urls-*.txt to full per-template URL sets
- representative pages (/ , /blog) unchanged; about-us + category untouched
- all 15 catalog pages now imported and previewing; 0 dropped source text

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article-listing.report.xlsx
+++ b/tools/importer/reports/import-article-listing.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="102">
   <si>
     <t>_reportFile</t>
   </si>
@@ -70,7 +70,7 @@
     <t>article-listing</t>
   </si>
   <si>
-    <t>2026-09-09T06:14:39.174Z</t>
+    <t>2026-09-09T10:46:04.718Z</t>
   </si>
   <si>
     <t>Blog — WKND Trendsetters</t>
@@ -79,19 +79,244 @@
     <t>https://wknd-trendsetters.site/blog</t>
   </si>
   <si>
+    <t>case-studies.report.json</t>
+  </si>
+  <si>
+    <t>["columns-intro","columns-article","cards-gallery","tabs-team","hero-overlay"]</t>
+  </si>
+  <si>
+    <t>case-studies</t>
+  </si>
+  <si>
+    <t>2026-09-09T10:46:10.251Z</t>
+  </si>
+  <si>
+    <t>Inspiring Case Studies | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/case-studies</t>
+  </si>
+  <si>
+    <t>faq.report.json</t>
+  </si>
+  <si>
+    <t>["columns-intro","columns-intro","accordion-faq"]</t>
+  </si>
+  <si>
+    <t>faq</t>
+  </si>
+  <si>
+    <t>faq-page</t>
+  </si>
+  <si>
+    <t>2026-09-09T06:28:00.720Z</t>
+  </si>
+  <si>
+    <t>FAQ - The Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/faq</t>
+  </si>
+  <si>
+    <t>fashion-insights.report.json</t>
+  </si>
+  <si>
+    <t>["columns-intro","columns-article","cards-article","cards-gallery"]</t>
+  </si>
+  <si>
+    <t>fashion-insights</t>
+  </si>
+  <si>
+    <t>2026-09-09T10:46:15.742Z</t>
+  </si>
+  <si>
+    <t>Fashion Blog - Discover Trends in Young Fashion</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/fashion-insights</t>
+  </si>
+  <si>
+    <t>fashion-trends-of-the-season.report.json</t>
+  </si>
+  <si>
+    <t>["columns-intro","columns-article","cards-gallery"]</t>
+  </si>
+  <si>
+    <t>fashion-trends-of-the-season</t>
+  </si>
+  <si>
+    <t>landing-page</t>
+  </si>
+  <si>
+    <t>2026-09-09T10:45:40.933Z</t>
+  </si>
+  <si>
+    <t>Top Fashion Trends for Young People | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/fashion-trends-of-the-season</t>
+  </si>
+  <si>
+    <t>fashion-trends-young-adults-casual-sport.report.json</t>
+  </si>
+  <si>
+    <t>["columns-intro","cards-trends","columns-article"]</t>
+  </si>
+  <si>
+    <t>fashion-trends-young-adults-casual-sport</t>
+  </si>
+  <si>
+    <t>category-collection</t>
+  </si>
+  <si>
+    <t>2026-09-09T07:03:53.840Z</t>
+  </si>
+  <si>
+    <t>Fashion Trends for Young Adults | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/fashion-trends-young-adults-casual-sport</t>
+  </si>
+  <si>
+    <t>fashion-trends-young-adults.report.json</t>
+  </si>
+  <si>
+    <t>["columns-intro","cards-gallery","cards-article"]</t>
+  </si>
+  <si>
+    <t>fashion-trends-young-adults</t>
+  </si>
+  <si>
+    <t>2026-09-09T10:45:44.352Z</t>
+  </si>
+  <si>
+    <t>Fashion Trends for Young Adults - Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/fashion-trends-young-adults</t>
+  </si>
+  <si>
     <t>index.report.json</t>
   </si>
   <si>
     <t>index</t>
   </si>
   <si>
-    <t>landing-page</t>
-  </si>
-  <si>
-    <t>2026-09-09T06:06:23.036Z</t>
+    <t>2026-09-09T10:45:35.169Z</t>
   </si>
   <si>
     <t>https://wknd-trendsetters.site/</t>
+  </si>
+  <si>
+    <t>blog/ace-pro-court-polo.report.json</t>
+  </si>
+  <si>
+    <t>["columns-article"]</t>
+  </si>
+  <si>
+    <t>blog/ace-pro-court-polo</t>
+  </si>
+  <si>
+    <t>blog-article</t>
+  </si>
+  <si>
+    <t>2026-09-09T06:19:57.450Z</t>
+  </si>
+  <si>
+    <t>Court cool, street ready — the Ace Pro polo | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/blog/ace-pro-court-polo</t>
+  </si>
+  <si>
+    <t>blog/fashion-blog-post.report.json</t>
+  </si>
+  <si>
+    <t>blog/fashion-blog-post</t>
+  </si>
+  <si>
+    <t>2026-09-09T10:27:08.366Z</t>
+  </si>
+  <si>
+    <t>Game on, style up | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/blog/fashion-blog-post</t>
+  </si>
+  <si>
+    <t>blog/fashion-trends-young-culture.report.json</t>
+  </si>
+  <si>
+    <t>blog/fashion-trends-young-culture</t>
+  </si>
+  <si>
+    <t>2026-09-09T10:27:12.619Z</t>
+  </si>
+  <si>
+    <t>Sunkissed and effortless | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/blog/fashion-trends-young-culture</t>
+  </si>
+  <si>
+    <t>blog/fashion-trends-young-style.report.json</t>
+  </si>
+  <si>
+    <t>blog/fashion-trends-young-style</t>
+  </si>
+  <si>
+    <t>2026-09-09T10:27:17.189Z</t>
+  </si>
+  <si>
+    <t>Party fits that pop | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/blog/fashion-trends-young-style</t>
+  </si>
+  <si>
+    <t>blog/flip-flop-summer-style.report.json</t>
+  </si>
+  <si>
+    <t>blog/flip-flop-summer-style</t>
+  </si>
+  <si>
+    <t>2026-09-09T10:27:21.495Z</t>
+  </si>
+  <si>
+    <t>Slide into summer — flip flops that serve | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/blog/flip-flop-summer-style</t>
+  </si>
+  <si>
+    <t>blog/latest-trends-young-casual-fashion.report.json</t>
+  </si>
+  <si>
+    <t>blog/latest-trends-young-casual-fashion</t>
+  </si>
+  <si>
+    <t>2026-09-09T10:27:26.894Z</t>
+  </si>
+  <si>
+    <t>Tennis style, redefined | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/blog/latest-trends-young-casual-fashion</t>
+  </si>
+  <si>
+    <t>blog/street-style-trends.report.json</t>
+  </si>
+  <si>
+    <t>blog/street-style-trends</t>
+  </si>
+  <si>
+    <t>2026-09-09T10:27:30.556Z</t>
+  </si>
+  <si>
+    <t>Street style, your way | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/blog/street-style-trends</t>
   </si>
 </sst>
 </file>
@@ -480,16 +705,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="42" customWidth="1"/>
+    <col min="5" max="5" width="21" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="41" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -575,25 +798,363 @@
         <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F4" t="s">
         <v>25</v>
       </c>
       <c r="G4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" t="s">
+        <v>46</v>
+      </c>
+      <c r="H7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>44</v>
+      </c>
+      <c r="F9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" t="s">
+        <v>59</v>
+      </c>
+      <c r="H9" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" t="s">
+        <v>63</v>
+      </c>
+      <c r="G10" t="s">
         <v>13</v>
       </c>
-      <c r="H4" t="s">
-        <v>26</v>
+      <c r="H10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>68</v>
+      </c>
+      <c r="F11" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" t="s">
+        <v>70</v>
+      </c>
+      <c r="H11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F12" t="s">
+        <v>74</v>
+      </c>
+      <c r="G12" t="s">
+        <v>75</v>
+      </c>
+      <c r="H12" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" t="s">
+        <v>78</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13" t="s">
+        <v>79</v>
+      </c>
+      <c r="G13" t="s">
+        <v>80</v>
+      </c>
+      <c r="H13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" t="s">
+        <v>83</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>68</v>
+      </c>
+      <c r="F14" t="s">
+        <v>84</v>
+      </c>
+      <c r="G14" t="s">
+        <v>85</v>
+      </c>
+      <c r="H14" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>87</v>
+      </c>
+      <c r="B15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" t="s">
+        <v>88</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>68</v>
+      </c>
+      <c r="F15" t="s">
+        <v>89</v>
+      </c>
+      <c r="G15" t="s">
+        <v>90</v>
+      </c>
+      <c r="H15" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>68</v>
+      </c>
+      <c r="F16" t="s">
+        <v>94</v>
+      </c>
+      <c r="G16" t="s">
+        <v>95</v>
+      </c>
+      <c r="H16" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" t="s">
+        <v>98</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>68</v>
+      </c>
+      <c r="F17" t="s">
+        <v>99</v>
+      </c>
+      <c r="G17" t="s">
+        <v>100</v>
+      </c>
+      <c r="H17" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>